<commit_message>
chore: update localization comparison results and synchronize backend string management scripts
</commit_message>
<xml_diff>
--- a/Python/Strings Comparer/ExcelData/picker-app-string.xlsx
+++ b/Python/Strings Comparer/ExcelData/picker-app-string.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="42" uniqueCount="31">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="93" uniqueCount="65">
   <si>
     <t>Key</t>
   </si>
@@ -104,6 +104,108 @@
   </si>
   <si>
     <t>description_qty</t>
+  </si>
+  <si>
+    <t>description_accepted</t>
+  </si>
+  <si>
+    <t>Accepted</t>
+  </si>
+  <si>
+    <t>description_doc_expired</t>
+  </si>
+  <si>
+    <t>Expired</t>
+  </si>
+  <si>
+    <t>description_heading_camera_permition_msg</t>
+  </si>
+  <si>
+    <t>To enhance your experience, we require access to your camera. Kindly allow camera permissions to continue.</t>
+  </si>
+  <si>
+    <t>description_hyperpay</t>
+  </si>
+  <si>
+    <t>Hyperpay</t>
+  </si>
+  <si>
+    <t>description_mercado_pago</t>
+  </si>
+  <si>
+    <t>Mercado Pago</t>
+  </si>
+  <si>
+    <t>description_mpesa</t>
+  </si>
+  <si>
+    <t>Mpesa</t>
+  </si>
+  <si>
+    <t>description_nestpay</t>
+  </si>
+  <si>
+    <t>NestPay</t>
+  </si>
+  <si>
+    <t>description_pago</t>
+  </si>
+  <si>
+    <t>Pago</t>
+  </si>
+  <si>
+    <t>description_paymob</t>
+  </si>
+  <si>
+    <t>Paymob</t>
+  </si>
+  <si>
+    <t>description_payu</t>
+  </si>
+  <si>
+    <t>PayU</t>
+  </si>
+  <si>
+    <t>description_pending</t>
+  </si>
+  <si>
+    <t>Pending</t>
+  </si>
+  <si>
+    <t>description_qicard</t>
+  </si>
+  <si>
+    <t>QiCard</t>
+  </si>
+  <si>
+    <t>description_rejected</t>
+  </si>
+  <si>
+    <t>Rejected</t>
+  </si>
+  <si>
+    <t>description_uploaded</t>
+  </si>
+  <si>
+    <t>Uploaded</t>
+  </si>
+  <si>
+    <t>description_zaincash</t>
+  </si>
+  <si>
+    <t>ZainCash</t>
+  </si>
+  <si>
+    <t>error_phone_not_valid</t>
+  </si>
+  <si>
+    <t>Please enter valid phone number</t>
+  </si>
+  <si>
+    <t>heading_camera_permition_alert</t>
+  </si>
+  <si>
+    <t>Camera Permission Required</t>
   </si>
 </sst>
 </file>
@@ -484,7 +586,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:I12"/>
+  <dimension ref="A1:I29"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="5" width="10" customWidth="1"/>
@@ -642,6 +744,193 @@
         <v>29</v>
       </c>
     </row>
+    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>31</v>
+      </c>
+      <c r="B13" t="s">
+        <v>10</v>
+      </c>
+      <c r="C13" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>33</v>
+      </c>
+      <c r="B14" t="s">
+        <v>10</v>
+      </c>
+      <c r="C14" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>35</v>
+      </c>
+      <c r="B15" t="s">
+        <v>10</v>
+      </c>
+      <c r="C15" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
+        <v>37</v>
+      </c>
+      <c r="B16" t="s">
+        <v>10</v>
+      </c>
+      <c r="C16" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
+        <v>39</v>
+      </c>
+      <c r="B17" t="s">
+        <v>10</v>
+      </c>
+      <c r="C17" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
+        <v>41</v>
+      </c>
+      <c r="B18" t="s">
+        <v>10</v>
+      </c>
+      <c r="C18" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
+        <v>43</v>
+      </c>
+      <c r="B19" t="s">
+        <v>10</v>
+      </c>
+      <c r="C19" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="20" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A20" t="s">
+        <v>45</v>
+      </c>
+      <c r="B20" t="s">
+        <v>10</v>
+      </c>
+      <c r="C20" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="21" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A21" t="s">
+        <v>47</v>
+      </c>
+      <c r="B21" t="s">
+        <v>10</v>
+      </c>
+      <c r="C21" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="22" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A22" t="s">
+        <v>49</v>
+      </c>
+      <c r="B22" t="s">
+        <v>10</v>
+      </c>
+      <c r="C22" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="23" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A23" t="s">
+        <v>51</v>
+      </c>
+      <c r="B23" t="s">
+        <v>10</v>
+      </c>
+      <c r="C23" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="24" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A24" t="s">
+        <v>53</v>
+      </c>
+      <c r="B24" t="s">
+        <v>10</v>
+      </c>
+      <c r="C24" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="25" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A25" t="s">
+        <v>55</v>
+      </c>
+      <c r="B25" t="s">
+        <v>10</v>
+      </c>
+      <c r="C25" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="26" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A26" t="s">
+        <v>57</v>
+      </c>
+      <c r="B26" t="s">
+        <v>10</v>
+      </c>
+      <c r="C26" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="27" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A27" t="s">
+        <v>59</v>
+      </c>
+      <c r="B27" t="s">
+        <v>10</v>
+      </c>
+      <c r="C27" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="28" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A28" t="s">
+        <v>61</v>
+      </c>
+      <c r="B28" t="s">
+        <v>10</v>
+      </c>
+      <c r="C28" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="29" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A29" t="s">
+        <v>63</v>
+      </c>
+      <c r="B29" t="s">
+        <v>10</v>
+      </c>
+      <c r="C29" t="s">
+        <v>64</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>

</xml_diff>